<commit_message>
repetetive requesting and sensor_data
</commit_message>
<xml_diff>
--- a/latest_response_data.xlsx
+++ b/latest_response_data.xlsx
@@ -458,11 +458,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>{'utc': '2026-01-09T16:00:00Z', 'local': '2026-01-09T09:00:00-07:00'}</t>
+          <t>{'utc': '2026-01-09T17:00:00Z', 'local': '2026-01-09T10:00:00-07:00'}</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.01</v>
+        <v>0.012</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -479,7 +479,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>{'utc': '2026-01-09T16:00:00Z', 'local': '2026-01-09T09:00:00-07:00'}</t>
+          <t>{'utc': '2026-01-09T17:00:00Z', 'local': '2026-01-09T10:00:00-07:00'}</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -500,7 +500,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>{'utc': '2026-01-09T16:00:00Z', 'local': '2026-01-09T09:00:00-07:00'}</t>
+          <t>{'utc': '2026-01-09T17:00:00Z', 'local': '2026-01-09T10:00:00-07:00'}</t>
         </is>
       </c>
       <c r="B4" t="n">
@@ -521,11 +521,11 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>{'utc': '2026-01-09T16:00:00Z', 'local': '2026-01-09T09:00:00-07:00'}</t>
+          <t>{'utc': '2026-01-09T17:00:00Z', 'local': '2026-01-09T10:00:00-07:00'}</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.034</v>
+        <v>0.036</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -542,11 +542,11 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>{'utc': '2026-01-09T16:00:00Z', 'local': '2026-01-09T09:00:00-07:00'}</t>
+          <t>{'utc': '2026-01-09T17:00:00Z', 'local': '2026-01-09T10:00:00-07:00'}</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -563,7 +563,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>{'utc': '2026-01-09T16:00:00Z', 'local': '2026-01-09T09:00:00-07:00'}</t>
+          <t>{'utc': '2026-01-09T17:00:00Z', 'local': '2026-01-09T10:00:00-07:00'}</t>
         </is>
       </c>
       <c r="B7" t="n">

</xml_diff>

<commit_message>
request_script complete: values and sensorID merged
</commit_message>
<xml_diff>
--- a/latest_response_data.xlsx
+++ b/latest_response_data.xlsx
@@ -458,11 +458,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>{'utc': '2026-01-09T17:00:00Z', 'local': '2026-01-09T10:00:00-07:00'}</t>
+          <t>{'utc': '2026-01-11T15:00:00Z', 'local': '2026-01-11T08:00:00-07:00'}</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.012</v>
+        <v>0.026</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -479,7 +479,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>{'utc': '2026-01-09T17:00:00Z', 'local': '2026-01-09T10:00:00-07:00'}</t>
+          <t>{'utc': '2026-01-11T15:00:00Z', 'local': '2026-01-11T08:00:00-07:00'}</t>
         </is>
       </c>
       <c r="B3" t="n">
@@ -500,11 +500,11 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>{'utc': '2026-01-09T17:00:00Z', 'local': '2026-01-09T10:00:00-07:00'}</t>
+          <t>{'utc': '2026-01-11T15:00:00Z', 'local': '2026-01-11T08:00:00-07:00'}</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2</v>
+        <v>5.3</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -521,11 +521,11 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>{'utc': '2026-01-09T17:00:00Z', 'local': '2026-01-09T10:00:00-07:00'}</t>
+          <t>{'utc': '2026-01-11T15:00:00Z', 'local': '2026-01-11T08:00:00-07:00'}</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.036</v>
+        <v>0.012</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -542,11 +542,11 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>{'utc': '2026-01-09T17:00:00Z', 'local': '2026-01-09T10:00:00-07:00'}</t>
+          <t>{'utc': '2026-01-11T15:00:00Z', 'local': '2026-01-11T08:00:00-07:00'}</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -563,11 +563,11 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>{'utc': '2026-01-09T17:00:00Z', 'local': '2026-01-09T10:00:00-07:00'}</t>
+          <t>{'utc': '2026-01-11T15:00:00Z', 'local': '2026-01-11T08:00:00-07:00'}</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
next: data_history and analysis
</commit_message>
<xml_diff>
--- a/latest_response_data.xlsx
+++ b/latest_response_data.xlsx
@@ -458,7 +458,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>{'utc': '2026-01-14T19:00:00Z', 'local': '2026-01-14T12:00:00-07:00'}</t>
+          <t>{'utc': '2026-01-14T20:00:00Z', 'local': '2026-01-14T13:00:00-07:00'}</t>
         </is>
       </c>
       <c r="B2" t="n">
@@ -500,11 +500,11 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>{'utc': '2026-01-14T19:00:00Z', 'local': '2026-01-14T12:00:00-07:00'}</t>
+          <t>{'utc': '2026-01-14T20:00:00Z', 'local': '2026-01-14T13:00:00-07:00'}</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>3.8</v>
+        <v>3.9</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -521,11 +521,11 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>{'utc': '2026-01-14T19:00:00Z', 'local': '2026-01-14T12:00:00-07:00'}</t>
+          <t>{'utc': '2026-01-14T20:00:00Z', 'local': '2026-01-14T13:00:00-07:00'}</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.03</v>
+        <v>0.033</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -542,11 +542,11 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>{'utc': '2026-01-14T19:00:00Z', 'local': '2026-01-14T12:00:00-07:00'}</t>
+          <t>{'utc': '2026-01-14T20:00:00Z', 'local': '2026-01-14T13:00:00-07:00'}</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -563,7 +563,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>{'utc': '2026-01-14T19:00:00Z', 'local': '2026-01-14T12:00:00-07:00'}</t>
+          <t>{'utc': '2026-01-14T20:00:00Z', 'local': '2026-01-14T13:00:00-07:00'}</t>
         </is>
       </c>
       <c r="B7" t="n">

</xml_diff>